<commit_message>
fix: add missing cadTrustUnitLabelId PK column to unitLabels sheet
</commit_message>
<xml_diff>
--- a/tests/v2/live-api/data/sample-units-import.xlsx
+++ b/tests/v2/live-api/data/sample-units-import.xlsx
@@ -677,53 +677,62 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>cadTrustUnitLabelId</v>
+      </c>
+      <c r="B1" t="str">
         <v>cadTrustLabelId</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
         <v>cadTrustUnitId</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>labelUnitDate</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>labelUnitDescription</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>NEW-1</v>
+      </c>
+      <c r="B2" t="str">
         <v>{{LABEL_ID}}</v>
       </c>
-      <c r="B2" t="str">
+      <c r="C2" t="str">
         <v>NEW-3</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>2024-06-15</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>Sample certification label — example description for unit testing</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>NEW-2</v>
+      </c>
+      <c r="B3" t="str">
         <v>{{LABEL_ID}}</v>
       </c>
-      <c r="B3" t="str">
+      <c r="C3" t="str">
         <v>NEW-4</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>2025-03-01</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>Sample authorized credit label — example description for unit testing</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: use distinct NEW-5/NEW-6 placeholders for unitLabel PKs
Avoids collision with UNIT_1/UNIT_2 (NEW-1/NEW-2) since
transformMetaUid performs global replacement within the same XLSX file.
</commit_message>
<xml_diff>
--- a/tests/v2/live-api/data/sample-units-import.xlsx
+++ b/tests/v2/live-api/data/sample-units-import.xlsx
@@ -698,7 +698,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>NEW-1</v>
+        <v>NEW-5</v>
       </c>
       <c r="B2" t="str">
         <v>{{LABEL_ID}}</v>
@@ -715,7 +715,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>NEW-2</v>
+        <v>NEW-6</v>
       </c>
       <c r="B3" t="str">
         <v>{{LABEL_ID}}</v>

</xml_diff>